<commit_message>
Update Gesss - 2026-09-18T04:52:23
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F56"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,13 +430,13 @@
         <v>SALDO INIZIALE</v>
       </c>
       <c r="D2">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E2" t="str">
         <v/>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>Utente: Gesss - Generato il 18/09/2026</v>
       </c>
     </row>
     <row r="3">
@@ -524,16 +524,16 @@
         <v>2026-08-21</v>
       </c>
       <c r="B7">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C7" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>154.07</v>
       </c>
       <c r="E7">
-        <v>-50</v>
+        <v>124.07</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -541,19 +541,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-08-21</v>
+        <v>2026-08-22</v>
       </c>
       <c r="B8">
         <v>30</v>
       </c>
       <c r="C8" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D8">
-        <v>154.07</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>124.07</v>
+        <v>-30</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -564,7 +564,7 @@
         <v>2026-08-22</v>
       </c>
       <c r="B9">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="C9" t="str">
         <v>Persa</v>
@@ -573,7 +573,7 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>-30</v>
+        <v>-6</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -584,7 +584,7 @@
         <v>2026-08-22</v>
       </c>
       <c r="B10">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C10" t="str">
         <v>Persa</v>
@@ -593,7 +593,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>-30</v>
+        <v>-100</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -601,10 +601,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-24</v>
       </c>
       <c r="B11">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="C11" t="str">
         <v>Persa</v>
@@ -613,7 +613,7 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>-6</v>
+        <v>-128</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -621,19 +621,19 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-28</v>
       </c>
       <c r="B12">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C12" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>339.6</v>
       </c>
       <c r="E12">
-        <v>-30</v>
+        <v>289.6</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -641,19 +641,19 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-28</v>
       </c>
       <c r="B13">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C13" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>386.58</v>
       </c>
       <c r="E13">
-        <v>-30</v>
+        <v>286.58</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -661,10 +661,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-28</v>
       </c>
       <c r="B14">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C14" t="str">
         <v>Persa</v>
@@ -673,7 +673,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -681,10 +681,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-28</v>
       </c>
       <c r="B15">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="C15" t="str">
         <v>Persa</v>
@@ -693,7 +693,7 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>-100</v>
+        <v>-30</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -701,10 +701,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-08-24</v>
+        <v>2026-08-29</v>
       </c>
       <c r="B16">
-        <v>128</v>
+        <v>50</v>
       </c>
       <c r="C16" t="str">
         <v>Persa</v>
@@ -713,7 +713,7 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-128</v>
+        <v>-50</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -721,19 +721,19 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-08-28</v>
+        <v>2026-08-29</v>
       </c>
       <c r="B17">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C17" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D17">
-        <v>339.6</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>289.6</v>
+        <v>-10</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -741,19 +741,19 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-08-28</v>
+        <v>2026-08-29</v>
       </c>
       <c r="B18">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C18" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D18">
-        <v>140.04</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>90.03999999999999</v>
+        <v>-55</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -761,19 +761,19 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-08-28</v>
+        <v>2026-08-31</v>
       </c>
       <c r="B19">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="C19" t="str">
         <v>Vinta</v>
       </c>
       <c r="D19">
-        <v>386.58</v>
+        <v>118.37</v>
       </c>
       <c r="E19">
-        <v>286.58</v>
+        <v>78.37</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -781,19 +781,19 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-08-28</v>
+        <v>2026-08-31</v>
       </c>
       <c r="B20">
         <v>50</v>
       </c>
       <c r="C20" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>299.52</v>
       </c>
       <c r="E20">
-        <v>-50</v>
+        <v>249.51999999999998</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -801,19 +801,19 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-01</v>
       </c>
       <c r="B21">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="C21" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>255.06</v>
       </c>
       <c r="E21">
-        <v>-30</v>
+        <v>175.06</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -821,19 +821,19 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-01</v>
       </c>
       <c r="B22">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="C22" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>247.25</v>
       </c>
       <c r="E22">
-        <v>-50</v>
+        <v>163.25</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -841,19 +841,19 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-02</v>
       </c>
       <c r="B23">
-        <v>50</v>
+        <v>160</v>
       </c>
       <c r="C23" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D23">
-        <v>164.35</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>114.35</v>
+        <v>-160</v>
       </c>
       <c r="F23" t="str">
         <v/>
@@ -861,7 +861,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-08-29</v>
+        <v>2026-09-02</v>
       </c>
       <c r="B24">
         <v>50</v>
@@ -881,10 +881,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-08-29</v>
+        <v>2026-09-03</v>
       </c>
       <c r="B25">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C25" t="str">
         <v>Persa</v>
@@ -893,7 +893,7 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>-10</v>
+        <v>-50</v>
       </c>
       <c r="F25" t="str">
         <v/>
@@ -901,7 +901,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-08-29</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B26">
         <v>50</v>
@@ -921,10 +921,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-08-29</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B27">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C27" t="str">
         <v>Persa</v>
@@ -933,7 +933,7 @@
         <v>0</v>
       </c>
       <c r="E27">
-        <v>-55</v>
+        <v>-42</v>
       </c>
       <c r="F27" t="str">
         <v/>
@@ -941,19 +941,19 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B28">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="C28" t="str">
         <v>Vinta</v>
       </c>
       <c r="D28">
-        <v>118.37</v>
+        <v>313.01</v>
       </c>
       <c r="E28">
-        <v>78.37</v>
+        <v>213.01</v>
       </c>
       <c r="F28" t="str">
         <v/>
@@ -961,19 +961,19 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B29">
         <v>50</v>
       </c>
       <c r="C29" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D29">
-        <v>299.52</v>
+        <v>0</v>
       </c>
       <c r="E29">
-        <v>249.51999999999998</v>
+        <v>-50</v>
       </c>
       <c r="F29" t="str">
         <v/>
@@ -981,19 +981,19 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-09-01</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B30">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="C30" t="str">
         <v>Vinta</v>
       </c>
       <c r="D30">
-        <v>255.06</v>
+        <v>190.68</v>
       </c>
       <c r="E30">
-        <v>175.06</v>
+        <v>140.68</v>
       </c>
       <c r="F30" t="str">
         <v/>
@@ -1001,19 +1001,19 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-09-01</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B31">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="C31" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D31">
-        <v>247.25</v>
+        <v>0</v>
       </c>
       <c r="E31">
-        <v>163.25</v>
+        <v>-100</v>
       </c>
       <c r="F31" t="str">
         <v/>
@@ -1021,19 +1021,19 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-09-02</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B32">
-        <v>160</v>
+        <v>41</v>
       </c>
       <c r="C32" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>223.76</v>
       </c>
       <c r="E32">
-        <v>-160</v>
+        <v>182.76</v>
       </c>
       <c r="F32" t="str">
         <v/>
@@ -1041,7 +1041,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-09-02</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B33">
         <v>50</v>
@@ -1061,10 +1061,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-09-03</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B34">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C34" t="str">
         <v>Persa</v>
@@ -1073,7 +1073,7 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>-50</v>
+        <v>-100</v>
       </c>
       <c r="F34" t="str">
         <v/>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B35">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C35" t="str">
         <v>Persa</v>
@@ -1093,7 +1093,7 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>-50</v>
+        <v>-20</v>
       </c>
       <c r="F35" t="str">
         <v/>
@@ -1101,19 +1101,19 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B36">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C36" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D36">
-        <v>0</v>
+        <v>299.84</v>
       </c>
       <c r="E36">
-        <v>-42</v>
+        <v>249.83999999999997</v>
       </c>
       <c r="F36" t="str">
         <v/>
@@ -1121,10 +1121,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B37">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C37" t="str">
         <v>Persa</v>
@@ -1133,7 +1133,7 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>-50</v>
+        <v>-54</v>
       </c>
       <c r="F37" t="str">
         <v/>
@@ -1141,19 +1141,19 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B38">
-        <v>100</v>
+        <v>183</v>
       </c>
       <c r="C38" t="str">
         <v>Vinta</v>
       </c>
       <c r="D38">
-        <v>313.01</v>
+        <v>521.55</v>
       </c>
       <c r="E38">
-        <v>213.01</v>
+        <v>338.54999999999995</v>
       </c>
       <c r="F38" t="str">
         <v/>
@@ -1161,7 +1161,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-08</v>
       </c>
       <c r="B39">
         <v>50</v>
@@ -1181,19 +1181,19 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B40">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C40" t="str">
         <v>Vinta</v>
       </c>
       <c r="D40">
-        <v>190.68</v>
+        <v>313.47</v>
       </c>
       <c r="E40">
-        <v>140.68</v>
+        <v>262.47</v>
       </c>
       <c r="F40" t="str">
         <v/>
@@ -1201,10 +1201,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B41">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="C41" t="str">
         <v>Persa</v>
@@ -1213,7 +1213,7 @@
         <v>0</v>
       </c>
       <c r="E41">
-        <v>-100</v>
+        <v>-45</v>
       </c>
       <c r="F41" t="str">
         <v/>
@@ -1221,19 +1221,19 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B42">
-        <v>41</v>
+        <v>128</v>
       </c>
       <c r="C42" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D42">
-        <v>223.76</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>182.76</v>
+        <v>-128</v>
       </c>
       <c r="F42" t="str">
         <v/>
@@ -1241,7 +1241,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B43">
         <v>50</v>
@@ -1261,19 +1261,19 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B44">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C44" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D44">
-        <v>0</v>
+        <v>167.62</v>
       </c>
       <c r="E44">
-        <v>-100</v>
+        <v>117.62</v>
       </c>
       <c r="F44" t="str">
         <v/>
@@ -1281,10 +1281,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B45">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C45" t="str">
         <v>Persa</v>
@@ -1293,7 +1293,7 @@
         <v>0</v>
       </c>
       <c r="E45">
-        <v>-20</v>
+        <v>-50</v>
       </c>
       <c r="F45" t="str">
         <v/>
@@ -1301,19 +1301,19 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B46">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C46" t="str">
         <v>Vinta</v>
       </c>
       <c r="D46">
-        <v>299.84</v>
+        <v>460.1</v>
       </c>
       <c r="E46">
-        <v>249.83999999999997</v>
+        <v>360.1</v>
       </c>
       <c r="F46" t="str">
         <v/>
@@ -1321,10 +1321,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B47">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C47" t="str">
         <v>Persa</v>
@@ -1333,7 +1333,7 @@
         <v>0</v>
       </c>
       <c r="E47">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="F47" t="str">
         <v/>
@@ -1341,10 +1341,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B48">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="C48" t="str">
         <v>Persa</v>
@@ -1353,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="E48">
-        <v>-54</v>
+        <v>-20</v>
       </c>
       <c r="F48" t="str">
         <v/>
@@ -1361,19 +1361,19 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B49">
-        <v>183</v>
+        <v>100</v>
       </c>
       <c r="C49" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D49">
-        <v>521.55</v>
+        <v>0</v>
       </c>
       <c r="E49">
-        <v>338.54999999999995</v>
+        <v>-100</v>
       </c>
       <c r="F49" t="str">
         <v/>
@@ -1381,10 +1381,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B50">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C50" t="str">
         <v>Persa</v>
@@ -1393,7 +1393,7 @@
         <v>0</v>
       </c>
       <c r="E50">
-        <v>-50</v>
+        <v>-20</v>
       </c>
       <c r="F50" t="str">
         <v/>
@@ -1401,10 +1401,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B51">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="C51" t="str">
         <v>Persa</v>
@@ -1413,7 +1413,7 @@
         <v>0</v>
       </c>
       <c r="E51">
-        <v>-50</v>
+        <v>-68</v>
       </c>
       <c r="F51" t="str">
         <v/>
@@ -1421,19 +1421,19 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B52">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C52" t="str">
         <v>Vinta</v>
       </c>
       <c r="D52">
-        <v>313.47</v>
+        <v>20.87</v>
       </c>
       <c r="E52">
-        <v>262.47</v>
+        <v>-29.13</v>
       </c>
       <c r="F52" t="str">
         <v/>
@@ -1441,10 +1441,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-15</v>
       </c>
       <c r="B53">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C53" t="str">
         <v>Persa</v>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="E53">
-        <v>-45</v>
+        <v>-44</v>
       </c>
       <c r="F53" t="str">
         <v/>
@@ -1461,10 +1461,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B54">
-        <v>128</v>
+        <v>50</v>
       </c>
       <c r="C54" t="str">
         <v>Persa</v>
@@ -1473,7 +1473,7 @@
         <v>0</v>
       </c>
       <c r="E54">
-        <v>-128</v>
+        <v>-50</v>
       </c>
       <c r="F54" t="str">
         <v/>
@@ -1481,19 +1481,19 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B55">
         <v>50</v>
       </c>
       <c r="C55" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D55">
-        <v>0</v>
+        <v>421.46</v>
       </c>
       <c r="E55">
-        <v>-50</v>
+        <v>371.46</v>
       </c>
       <c r="F55" t="str">
         <v/>
@@ -1501,387 +1501,27 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B56">
-        <v>50</v>
+        <v>170</v>
       </c>
       <c r="C56" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D56">
-        <v>167.62</v>
+        <v>0</v>
       </c>
       <c r="E56">
-        <v>117.62</v>
+        <v>-170</v>
       </c>
       <c r="F56" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>2026-09-11</v>
-      </c>
-      <c r="B57">
-        <v>50</v>
-      </c>
-      <c r="C57" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D57">
-        <v>0</v>
-      </c>
-      <c r="E57">
-        <v>-50</v>
-      </c>
-      <c r="F57" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>2026-09-11</v>
-      </c>
-      <c r="B58">
-        <v>50</v>
-      </c>
-      <c r="C58" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D58">
-        <v>0</v>
-      </c>
-      <c r="E58">
-        <v>-50</v>
-      </c>
-      <c r="F58" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>2026-09-11</v>
-      </c>
-      <c r="B59">
-        <v>50</v>
-      </c>
-      <c r="C59" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D59">
-        <v>0</v>
-      </c>
-      <c r="E59">
-        <v>-50</v>
-      </c>
-      <c r="F59" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>2026-09-11</v>
-      </c>
-      <c r="B60">
-        <v>100</v>
-      </c>
-      <c r="C60" t="str">
-        <v>Vinta</v>
-      </c>
-      <c r="D60">
-        <v>460.1</v>
-      </c>
-      <c r="E60">
-        <v>360.1</v>
-      </c>
-      <c r="F60" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B61">
-        <v>50</v>
-      </c>
-      <c r="C61" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D61">
-        <v>0</v>
-      </c>
-      <c r="E61">
-        <v>-50</v>
-      </c>
-      <c r="F61" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B62">
-        <v>50</v>
-      </c>
-      <c r="C62" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D62">
-        <v>0</v>
-      </c>
-      <c r="E62">
-        <v>-50</v>
-      </c>
-      <c r="F62" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B63">
-        <v>20</v>
-      </c>
-      <c r="C63" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D63">
-        <v>0</v>
-      </c>
-      <c r="E63">
-        <v>-20</v>
-      </c>
-      <c r="F63" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B64">
-        <v>50</v>
-      </c>
-      <c r="C64" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D64">
-        <v>0</v>
-      </c>
-      <c r="E64">
-        <v>-50</v>
-      </c>
-      <c r="F64" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B65">
-        <v>20</v>
-      </c>
-      <c r="C65" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D65">
-        <v>0</v>
-      </c>
-      <c r="E65">
-        <v>-20</v>
-      </c>
-      <c r="F65" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="str">
-        <v>2026-09-13</v>
-      </c>
-      <c r="B66">
-        <v>100</v>
-      </c>
-      <c r="C66" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D66">
-        <v>0</v>
-      </c>
-      <c r="E66">
-        <v>-100</v>
-      </c>
-      <c r="F66" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="str">
-        <v>2026-09-13</v>
-      </c>
-      <c r="B67">
-        <v>20</v>
-      </c>
-      <c r="C67" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D67">
-        <v>0</v>
-      </c>
-      <c r="E67">
-        <v>-20</v>
-      </c>
-      <c r="F67" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="str">
-        <v>2026-09-13</v>
-      </c>
-      <c r="B68">
-        <v>100</v>
-      </c>
-      <c r="C68" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D68">
-        <v>0</v>
-      </c>
-      <c r="E68">
-        <v>-100</v>
-      </c>
-      <c r="F68" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="str">
-        <v>2026-09-14</v>
-      </c>
-      <c r="B69">
-        <v>68</v>
-      </c>
-      <c r="C69" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D69">
-        <v>0</v>
-      </c>
-      <c r="E69">
-        <v>-68</v>
-      </c>
-      <c r="F69" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="str">
-        <v>2026-09-14</v>
-      </c>
-      <c r="B70">
-        <v>50</v>
-      </c>
-      <c r="C70" t="str">
-        <v>Vinta</v>
-      </c>
-      <c r="D70">
-        <v>20.87</v>
-      </c>
-      <c r="E70">
-        <v>-29.13</v>
-      </c>
-      <c r="F70" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="str">
-        <v>2026-09-15</v>
-      </c>
-      <c r="B71">
-        <v>44</v>
-      </c>
-      <c r="C71" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D71">
-        <v>0</v>
-      </c>
-      <c r="E71">
-        <v>-44</v>
-      </c>
-      <c r="F71" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="str">
-        <v>2026-09-16</v>
-      </c>
-      <c r="B72">
-        <v>50</v>
-      </c>
-      <c r="C72" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D72">
-        <v>0</v>
-      </c>
-      <c r="E72">
-        <v>-50</v>
-      </c>
-      <c r="F72" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="str">
-        <v>2026-09-17</v>
-      </c>
-      <c r="B73">
-        <v>50</v>
-      </c>
-      <c r="C73" t="str">
-        <v>Vinta</v>
-      </c>
-      <c r="D73">
-        <v>421.46</v>
-      </c>
-      <c r="E73">
-        <v>371.46</v>
-      </c>
-      <c r="F73" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="str">
-        <v>2026-09-17</v>
-      </c>
-      <c r="B74">
-        <v>170</v>
-      </c>
-      <c r="C74" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D74">
-        <v>0</v>
-      </c>
-      <c r="E74">
-        <v>-170</v>
-      </c>
-      <c r="F74" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F56"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-18T20:48:01
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F59"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1519,9 +1519,69 @@
         <v/>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B57">
+        <v>50</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Vinta</v>
+      </c>
+      <c r="D57">
+        <v>266.62</v>
+      </c>
+      <c r="E57">
+        <v>216.62</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B58">
+        <v>50</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D58">
+        <v>0</v>
+      </c>
+      <c r="E58">
+        <v>-50</v>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>2026-09-18</v>
+      </c>
+      <c r="B59">
+        <v>52</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D59">
+        <v>0</v>
+      </c>
+      <c r="E59">
+        <v>-52</v>
+      </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F59"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-19T07:24:36
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F59"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,13 +430,13 @@
         <v>SALDO INIZIALE</v>
       </c>
       <c r="D2">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="E2" t="str">
         <v/>
       </c>
       <c r="F2" t="str">
-        <v/>
+        <v>Utente: Gesss - Generato il 19/09/2026</v>
       </c>
     </row>
     <row r="3">
@@ -524,16 +524,16 @@
         <v>2026-08-21</v>
       </c>
       <c r="B7">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C7" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>154.07</v>
       </c>
       <c r="E7">
-        <v>-50</v>
+        <v>124.07</v>
       </c>
       <c r="F7" t="str">
         <v/>
@@ -541,19 +541,19 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2026-08-21</v>
+        <v>2026-08-22</v>
       </c>
       <c r="B8">
         <v>30</v>
       </c>
       <c r="C8" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D8">
-        <v>154.07</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>124.07</v>
+        <v>-30</v>
       </c>
       <c r="F8" t="str">
         <v/>
@@ -564,7 +564,7 @@
         <v>2026-08-22</v>
       </c>
       <c r="B9">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="C9" t="str">
         <v>Persa</v>
@@ -573,7 +573,7 @@
         <v>0</v>
       </c>
       <c r="E9">
-        <v>-30</v>
+        <v>-6</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -584,7 +584,7 @@
         <v>2026-08-22</v>
       </c>
       <c r="B10">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C10" t="str">
         <v>Persa</v>
@@ -593,7 +593,7 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>-30</v>
+        <v>-100</v>
       </c>
       <c r="F10" t="str">
         <v/>
@@ -601,10 +601,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-24</v>
       </c>
       <c r="B11">
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="C11" t="str">
         <v>Persa</v>
@@ -613,7 +613,7 @@
         <v>0</v>
       </c>
       <c r="E11">
-        <v>-6</v>
+        <v>-128</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -621,19 +621,19 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-28</v>
       </c>
       <c r="B12">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="C12" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>339.6</v>
       </c>
       <c r="E12">
-        <v>-30</v>
+        <v>289.6</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -641,19 +641,19 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-28</v>
       </c>
       <c r="B13">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C13" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>386.58</v>
       </c>
       <c r="E13">
-        <v>-30</v>
+        <v>286.58</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -661,10 +661,10 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-28</v>
       </c>
       <c r="B14">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C14" t="str">
         <v>Persa</v>
@@ -673,7 +673,7 @@
         <v>0</v>
       </c>
       <c r="E14">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="F14" t="str">
         <v/>
@@ -681,10 +681,10 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>2026-08-22</v>
+        <v>2026-08-28</v>
       </c>
       <c r="B15">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="C15" t="str">
         <v>Persa</v>
@@ -693,7 +693,7 @@
         <v>0</v>
       </c>
       <c r="E15">
-        <v>-100</v>
+        <v>-30</v>
       </c>
       <c r="F15" t="str">
         <v/>
@@ -701,10 +701,10 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-08-24</v>
+        <v>2026-08-29</v>
       </c>
       <c r="B16">
-        <v>128</v>
+        <v>50</v>
       </c>
       <c r="C16" t="str">
         <v>Persa</v>
@@ -713,7 +713,7 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <v>-128</v>
+        <v>-50</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -721,19 +721,19 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-08-28</v>
+        <v>2026-08-29</v>
       </c>
       <c r="B17">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C17" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D17">
-        <v>339.6</v>
+        <v>0</v>
       </c>
       <c r="E17">
-        <v>289.6</v>
+        <v>-10</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -741,19 +741,19 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-08-28</v>
+        <v>2026-08-29</v>
       </c>
       <c r="B18">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C18" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D18">
-        <v>140.04</v>
+        <v>0</v>
       </c>
       <c r="E18">
-        <v>90.03999999999999</v>
+        <v>-55</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -761,19 +761,19 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-08-28</v>
+        <v>2026-08-31</v>
       </c>
       <c r="B19">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="C19" t="str">
         <v>Vinta</v>
       </c>
       <c r="D19">
-        <v>386.58</v>
+        <v>118.37</v>
       </c>
       <c r="E19">
-        <v>286.58</v>
+        <v>78.37</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -781,19 +781,19 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-08-28</v>
+        <v>2026-08-31</v>
       </c>
       <c r="B20">
         <v>50</v>
       </c>
       <c r="C20" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D20">
-        <v>0</v>
+        <v>299.52</v>
       </c>
       <c r="E20">
-        <v>-50</v>
+        <v>249.51999999999998</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -801,19 +801,19 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-01</v>
       </c>
       <c r="B21">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="C21" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D21">
-        <v>0</v>
+        <v>255.06</v>
       </c>
       <c r="E21">
-        <v>-30</v>
+        <v>175.06</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -821,19 +821,19 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-01</v>
       </c>
       <c r="B22">
-        <v>50</v>
+        <v>84</v>
       </c>
       <c r="C22" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>247.25</v>
       </c>
       <c r="E22">
-        <v>-50</v>
+        <v>163.25</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -841,19 +841,19 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-08-28</v>
+        <v>2026-09-02</v>
       </c>
       <c r="B23">
-        <v>50</v>
+        <v>160</v>
       </c>
       <c r="C23" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D23">
-        <v>164.35</v>
+        <v>0</v>
       </c>
       <c r="E23">
-        <v>114.35</v>
+        <v>-160</v>
       </c>
       <c r="F23" t="str">
         <v/>
@@ -861,7 +861,7 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-08-29</v>
+        <v>2026-09-02</v>
       </c>
       <c r="B24">
         <v>50</v>
@@ -881,10 +881,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-08-29</v>
+        <v>2026-09-03</v>
       </c>
       <c r="B25">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C25" t="str">
         <v>Persa</v>
@@ -893,7 +893,7 @@
         <v>0</v>
       </c>
       <c r="E25">
-        <v>-10</v>
+        <v>-50</v>
       </c>
       <c r="F25" t="str">
         <v/>
@@ -901,7 +901,7 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-08-29</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B26">
         <v>50</v>
@@ -921,10 +921,10 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-08-29</v>
+        <v>2026-09-04</v>
       </c>
       <c r="B27">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C27" t="str">
         <v>Persa</v>
@@ -933,7 +933,7 @@
         <v>0</v>
       </c>
       <c r="E27">
-        <v>-55</v>
+        <v>-42</v>
       </c>
       <c r="F27" t="str">
         <v/>
@@ -941,19 +941,19 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B28">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="C28" t="str">
         <v>Vinta</v>
       </c>
       <c r="D28">
-        <v>118.37</v>
+        <v>313.01</v>
       </c>
       <c r="E28">
-        <v>78.37</v>
+        <v>213.01</v>
       </c>
       <c r="F28" t="str">
         <v/>
@@ -961,19 +961,19 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-08-31</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B29">
         <v>50</v>
       </c>
       <c r="C29" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D29">
-        <v>299.52</v>
+        <v>0</v>
       </c>
       <c r="E29">
-        <v>249.51999999999998</v>
+        <v>-50</v>
       </c>
       <c r="F29" t="str">
         <v/>
@@ -981,19 +981,19 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>2026-09-01</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B30">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="C30" t="str">
         <v>Vinta</v>
       </c>
       <c r="D30">
-        <v>255.06</v>
+        <v>190.68</v>
       </c>
       <c r="E30">
-        <v>175.06</v>
+        <v>140.68</v>
       </c>
       <c r="F30" t="str">
         <v/>
@@ -1001,19 +1001,19 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>2026-09-01</v>
+        <v>2026-09-05</v>
       </c>
       <c r="B31">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="C31" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D31">
-        <v>247.25</v>
+        <v>0</v>
       </c>
       <c r="E31">
-        <v>163.25</v>
+        <v>-100</v>
       </c>
       <c r="F31" t="str">
         <v/>
@@ -1021,19 +1021,19 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>2026-09-02</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B32">
-        <v>160</v>
+        <v>41</v>
       </c>
       <c r="C32" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D32">
-        <v>0</v>
+        <v>223.76</v>
       </c>
       <c r="E32">
-        <v>-160</v>
+        <v>182.76</v>
       </c>
       <c r="F32" t="str">
         <v/>
@@ -1041,7 +1041,7 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>2026-09-02</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B33">
         <v>50</v>
@@ -1061,10 +1061,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>2026-09-03</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B34">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C34" t="str">
         <v>Persa</v>
@@ -1073,7 +1073,7 @@
         <v>0</v>
       </c>
       <c r="E34">
-        <v>-50</v>
+        <v>-100</v>
       </c>
       <c r="F34" t="str">
         <v/>
@@ -1081,10 +1081,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B35">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C35" t="str">
         <v>Persa</v>
@@ -1093,7 +1093,7 @@
         <v>0</v>
       </c>
       <c r="E35">
-        <v>-50</v>
+        <v>-20</v>
       </c>
       <c r="F35" t="str">
         <v/>
@@ -1101,19 +1101,19 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-06</v>
       </c>
       <c r="B36">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="C36" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D36">
-        <v>0</v>
+        <v>299.84</v>
       </c>
       <c r="E36">
-        <v>-42</v>
+        <v>249.83999999999997</v>
       </c>
       <c r="F36" t="str">
         <v/>
@@ -1121,10 +1121,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>2026-09-04</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B37">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="C37" t="str">
         <v>Persa</v>
@@ -1133,7 +1133,7 @@
         <v>0</v>
       </c>
       <c r="E37">
-        <v>-50</v>
+        <v>-54</v>
       </c>
       <c r="F37" t="str">
         <v/>
@@ -1141,19 +1141,19 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-07</v>
       </c>
       <c r="B38">
-        <v>100</v>
+        <v>183</v>
       </c>
       <c r="C38" t="str">
         <v>Vinta</v>
       </c>
       <c r="D38">
-        <v>313.01</v>
+        <v>521.55</v>
       </c>
       <c r="E38">
-        <v>213.01</v>
+        <v>338.54999999999995</v>
       </c>
       <c r="F38" t="str">
         <v/>
@@ -1161,7 +1161,7 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-08</v>
       </c>
       <c r="B39">
         <v>50</v>
@@ -1181,19 +1181,19 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B40">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C40" t="str">
         <v>Vinta</v>
       </c>
       <c r="D40">
-        <v>190.68</v>
+        <v>313.47</v>
       </c>
       <c r="E40">
-        <v>140.68</v>
+        <v>262.47</v>
       </c>
       <c r="F40" t="str">
         <v/>
@@ -1201,10 +1201,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>2026-09-05</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B41">
-        <v>100</v>
+        <v>45</v>
       </c>
       <c r="C41" t="str">
         <v>Persa</v>
@@ -1213,7 +1213,7 @@
         <v>0</v>
       </c>
       <c r="E41">
-        <v>-100</v>
+        <v>-45</v>
       </c>
       <c r="F41" t="str">
         <v/>
@@ -1221,19 +1221,19 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-09</v>
       </c>
       <c r="B42">
-        <v>41</v>
+        <v>128</v>
       </c>
       <c r="C42" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D42">
-        <v>223.76</v>
+        <v>0</v>
       </c>
       <c r="E42">
-        <v>182.76</v>
+        <v>-128</v>
       </c>
       <c r="F42" t="str">
         <v/>
@@ -1241,7 +1241,7 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B43">
         <v>50</v>
@@ -1261,19 +1261,19 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-10</v>
       </c>
       <c r="B44">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C44" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D44">
-        <v>0</v>
+        <v>167.62</v>
       </c>
       <c r="E44">
-        <v>-100</v>
+        <v>117.62</v>
       </c>
       <c r="F44" t="str">
         <v/>
@@ -1281,10 +1281,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B45">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C45" t="str">
         <v>Persa</v>
@@ -1293,7 +1293,7 @@
         <v>0</v>
       </c>
       <c r="E45">
-        <v>-20</v>
+        <v>-50</v>
       </c>
       <c r="F45" t="str">
         <v/>
@@ -1301,19 +1301,19 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-11</v>
       </c>
       <c r="B46">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C46" t="str">
         <v>Vinta</v>
       </c>
       <c r="D46">
-        <v>299.84</v>
+        <v>460.1</v>
       </c>
       <c r="E46">
-        <v>249.83999999999997</v>
+        <v>360.1</v>
       </c>
       <c r="F46" t="str">
         <v/>
@@ -1321,10 +1321,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>2026-09-06</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B47">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C47" t="str">
         <v>Persa</v>
@@ -1333,7 +1333,7 @@
         <v>0</v>
       </c>
       <c r="E47">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="F47" t="str">
         <v/>
@@ -1341,10 +1341,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-12</v>
       </c>
       <c r="B48">
-        <v>54</v>
+        <v>20</v>
       </c>
       <c r="C48" t="str">
         <v>Persa</v>
@@ -1353,7 +1353,7 @@
         <v>0</v>
       </c>
       <c r="E48">
-        <v>-54</v>
+        <v>-20</v>
       </c>
       <c r="F48" t="str">
         <v/>
@@ -1361,19 +1361,19 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>2026-09-07</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B49">
-        <v>183</v>
+        <v>100</v>
       </c>
       <c r="C49" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D49">
-        <v>521.55</v>
+        <v>0</v>
       </c>
       <c r="E49">
-        <v>338.54999999999995</v>
+        <v>-100</v>
       </c>
       <c r="F49" t="str">
         <v/>
@@ -1381,10 +1381,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-13</v>
       </c>
       <c r="B50">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C50" t="str">
         <v>Persa</v>
@@ -1393,7 +1393,7 @@
         <v>0</v>
       </c>
       <c r="E50">
-        <v>-50</v>
+        <v>-20</v>
       </c>
       <c r="F50" t="str">
         <v/>
@@ -1401,10 +1401,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>2026-09-08</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B51">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="C51" t="str">
         <v>Persa</v>
@@ -1413,7 +1413,7 @@
         <v>0</v>
       </c>
       <c r="E51">
-        <v>-50</v>
+        <v>-68</v>
       </c>
       <c r="F51" t="str">
         <v/>
@@ -1421,19 +1421,19 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-14</v>
       </c>
       <c r="B52">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C52" t="str">
         <v>Vinta</v>
       </c>
       <c r="D52">
-        <v>313.47</v>
+        <v>20.87</v>
       </c>
       <c r="E52">
-        <v>262.47</v>
+        <v>-29.13</v>
       </c>
       <c r="F52" t="str">
         <v/>
@@ -1441,10 +1441,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-15</v>
       </c>
       <c r="B53">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C53" t="str">
         <v>Persa</v>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="E53">
-        <v>-45</v>
+        <v>-44</v>
       </c>
       <c r="F53" t="str">
         <v/>
@@ -1461,10 +1461,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>2026-09-09</v>
+        <v>2026-09-16</v>
       </c>
       <c r="B54">
-        <v>128</v>
+        <v>50</v>
       </c>
       <c r="C54" t="str">
         <v>Persa</v>
@@ -1473,7 +1473,7 @@
         <v>0</v>
       </c>
       <c r="E54">
-        <v>-128</v>
+        <v>-50</v>
       </c>
       <c r="F54" t="str">
         <v/>
@@ -1481,19 +1481,19 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B55">
         <v>50</v>
       </c>
       <c r="C55" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D55">
-        <v>0</v>
+        <v>421.46</v>
       </c>
       <c r="E55">
-        <v>-50</v>
+        <v>371.46</v>
       </c>
       <c r="F55" t="str">
         <v/>
@@ -1501,19 +1501,19 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>2026-09-10</v>
+        <v>2026-09-17</v>
       </c>
       <c r="B56">
-        <v>50</v>
+        <v>170</v>
       </c>
       <c r="C56" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D56">
-        <v>167.62</v>
+        <v>0</v>
       </c>
       <c r="E56">
-        <v>117.62</v>
+        <v>-170</v>
       </c>
       <c r="F56" t="str">
         <v/>
@@ -1521,19 +1521,19 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-18</v>
       </c>
       <c r="B57">
         <v>50</v>
       </c>
       <c r="C57" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D57">
-        <v>0</v>
+        <v>266.62</v>
       </c>
       <c r="E57">
-        <v>-50</v>
+        <v>216.62</v>
       </c>
       <c r="F57" t="str">
         <v/>
@@ -1541,7 +1541,7 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-18</v>
       </c>
       <c r="B58">
         <v>50</v>
@@ -1561,10 +1561,10 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>2026-09-11</v>
+        <v>2026-09-18</v>
       </c>
       <c r="B59">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C59" t="str">
         <v>Persa</v>
@@ -1573,315 +1573,15 @@
         <v>0</v>
       </c>
       <c r="E59">
-        <v>-50</v>
+        <v>-52</v>
       </c>
       <c r="F59" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>2026-09-11</v>
-      </c>
-      <c r="B60">
-        <v>100</v>
-      </c>
-      <c r="C60" t="str">
-        <v>Vinta</v>
-      </c>
-      <c r="D60">
-        <v>460.1</v>
-      </c>
-      <c r="E60">
-        <v>360.1</v>
-      </c>
-      <c r="F60" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B61">
-        <v>50</v>
-      </c>
-      <c r="C61" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D61">
-        <v>0</v>
-      </c>
-      <c r="E61">
-        <v>-50</v>
-      </c>
-      <c r="F61" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B62">
-        <v>50</v>
-      </c>
-      <c r="C62" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D62">
-        <v>0</v>
-      </c>
-      <c r="E62">
-        <v>-50</v>
-      </c>
-      <c r="F62" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B63">
-        <v>20</v>
-      </c>
-      <c r="C63" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D63">
-        <v>0</v>
-      </c>
-      <c r="E63">
-        <v>-20</v>
-      </c>
-      <c r="F63" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B64">
-        <v>50</v>
-      </c>
-      <c r="C64" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D64">
-        <v>0</v>
-      </c>
-      <c r="E64">
-        <v>-50</v>
-      </c>
-      <c r="F64" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="str">
-        <v>2026-09-12</v>
-      </c>
-      <c r="B65">
-        <v>20</v>
-      </c>
-      <c r="C65" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D65">
-        <v>0</v>
-      </c>
-      <c r="E65">
-        <v>-20</v>
-      </c>
-      <c r="F65" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="str">
-        <v>2026-09-13</v>
-      </c>
-      <c r="B66">
-        <v>100</v>
-      </c>
-      <c r="C66" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D66">
-        <v>0</v>
-      </c>
-      <c r="E66">
-        <v>-100</v>
-      </c>
-      <c r="F66" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="str">
-        <v>2026-09-13</v>
-      </c>
-      <c r="B67">
-        <v>20</v>
-      </c>
-      <c r="C67" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D67">
-        <v>0</v>
-      </c>
-      <c r="E67">
-        <v>-20</v>
-      </c>
-      <c r="F67" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="str">
-        <v>2026-09-13</v>
-      </c>
-      <c r="B68">
-        <v>100</v>
-      </c>
-      <c r="C68" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D68">
-        <v>0</v>
-      </c>
-      <c r="E68">
-        <v>-100</v>
-      </c>
-      <c r="F68" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="str">
-        <v>2026-09-14</v>
-      </c>
-      <c r="B69">
-        <v>68</v>
-      </c>
-      <c r="C69" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D69">
-        <v>0</v>
-      </c>
-      <c r="E69">
-        <v>-68</v>
-      </c>
-      <c r="F69" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="str">
-        <v>2026-09-14</v>
-      </c>
-      <c r="B70">
-        <v>50</v>
-      </c>
-      <c r="C70" t="str">
-        <v>Vinta</v>
-      </c>
-      <c r="D70">
-        <v>20.87</v>
-      </c>
-      <c r="E70">
-        <v>-29.13</v>
-      </c>
-      <c r="F70" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="str">
-        <v>2026-09-15</v>
-      </c>
-      <c r="B71">
-        <v>44</v>
-      </c>
-      <c r="C71" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D71">
-        <v>0</v>
-      </c>
-      <c r="E71">
-        <v>-44</v>
-      </c>
-      <c r="F71" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="str">
-        <v>2026-09-16</v>
-      </c>
-      <c r="B72">
-        <v>50</v>
-      </c>
-      <c r="C72" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D72">
-        <v>0</v>
-      </c>
-      <c r="E72">
-        <v>-50</v>
-      </c>
-      <c r="F72" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="str">
-        <v>2026-09-17</v>
-      </c>
-      <c r="B73">
-        <v>50</v>
-      </c>
-      <c r="C73" t="str">
-        <v>Vinta</v>
-      </c>
-      <c r="D73">
-        <v>421.46</v>
-      </c>
-      <c r="E73">
-        <v>371.46</v>
-      </c>
-      <c r="F73" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="str">
-        <v>2026-09-17</v>
-      </c>
-      <c r="B74">
-        <v>170</v>
-      </c>
-      <c r="C74" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D74">
-        <v>0</v>
-      </c>
-      <c r="E74">
-        <v>-170</v>
-      </c>
-      <c r="F74" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F59"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-21T19:21:59
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F67"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 19/09/2026</v>
+        <v>Utente: Gesss - Generato il 21/09/2026</v>
       </c>
     </row>
     <row r="3">
@@ -1579,9 +1579,169 @@
         <v/>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B60">
+        <v>50</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D60">
+        <v>0</v>
+      </c>
+      <c r="E60">
+        <v>-50</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B61">
+        <v>50</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D61">
+        <v>0</v>
+      </c>
+      <c r="E61">
+        <v>-50</v>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2026-09-19</v>
+      </c>
+      <c r="B62">
+        <v>100</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D62">
+        <v>0</v>
+      </c>
+      <c r="E62">
+        <v>-100</v>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B63">
+        <v>50</v>
+      </c>
+      <c r="C63" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D63">
+        <v>0</v>
+      </c>
+      <c r="E63">
+        <v>-50</v>
+      </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B64">
+        <v>50</v>
+      </c>
+      <c r="C64" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D64">
+        <v>0</v>
+      </c>
+      <c r="E64">
+        <v>-50</v>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B65">
+        <v>50</v>
+      </c>
+      <c r="C65" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D65">
+        <v>0</v>
+      </c>
+      <c r="E65">
+        <v>-50</v>
+      </c>
+      <c r="F65" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B66">
+        <v>50</v>
+      </c>
+      <c r="C66" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D66">
+        <v>0</v>
+      </c>
+      <c r="E66">
+        <v>-50</v>
+      </c>
+      <c r="F66" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-09-20</v>
+      </c>
+      <c r="B67">
+        <v>50</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D67">
+        <v>0</v>
+      </c>
+      <c r="E67">
+        <v>-50</v>
+      </c>
+      <c r="F67" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F59"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F67"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-21T20:31:30
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F67"/>
+  <dimension ref="A1:F69"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1739,9 +1739,49 @@
         <v/>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B68">
+        <v>66</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D68">
+        <v>0</v>
+      </c>
+      <c r="E68">
+        <v>-66</v>
+      </c>
+      <c r="F68" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>2026-09-21</v>
+      </c>
+      <c r="B69">
+        <v>200</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Vinta</v>
+      </c>
+      <c r="D69">
+        <v>598.16</v>
+      </c>
+      <c r="E69">
+        <v>398.15999999999997</v>
+      </c>
+      <c r="F69" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F67"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F69"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-25T18:00:14
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 21/09/2026</v>
+        <v>Utente: Gesss - Generato il 25/09/2026</v>
       </c>
     </row>
     <row r="3">
@@ -1779,9 +1779,29 @@
         <v/>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>2026-09-25</v>
+      </c>
+      <c r="B70">
+        <v>50</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D70">
+        <v>0</v>
+      </c>
+      <c r="E70">
+        <v>-50</v>
+      </c>
+      <c r="F70" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F69"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F70"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-26T06:25:47
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F70"/>
+  <dimension ref="A1:F73"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 25/09/2026</v>
+        <v>Utente: Gesss - Generato il 26/09/2026</v>
       </c>
     </row>
     <row r="3">
@@ -1799,9 +1799,69 @@
         <v/>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>2026-09-25</v>
+      </c>
+      <c r="B71">
+        <v>50</v>
+      </c>
+      <c r="C71" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D71">
+        <v>0</v>
+      </c>
+      <c r="E71">
+        <v>-50</v>
+      </c>
+      <c r="F71" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>2026-09-25</v>
+      </c>
+      <c r="B72">
+        <v>50</v>
+      </c>
+      <c r="C72" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D72">
+        <v>0</v>
+      </c>
+      <c r="E72">
+        <v>-50</v>
+      </c>
+      <c r="F72" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>2026-09-25</v>
+      </c>
+      <c r="B73">
+        <v>100</v>
+      </c>
+      <c r="C73" t="str">
+        <v>Vinta</v>
+      </c>
+      <c r="D73">
+        <v>172</v>
+      </c>
+      <c r="E73">
+        <v>72</v>
+      </c>
+      <c r="F73" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F73"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-26T20:40:06
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F75"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1824,16 +1824,16 @@
         <v>2026-09-25</v>
       </c>
       <c r="B72">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C72" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D72">
-        <v>0</v>
+        <v>172</v>
       </c>
       <c r="E72">
-        <v>-50</v>
+        <v>72</v>
       </c>
       <c r="F72" t="str">
         <v/>
@@ -1841,27 +1841,67 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-09-25</v>
+        <v>2026-09-26</v>
       </c>
       <c r="B73">
         <v>100</v>
       </c>
       <c r="C73" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D73">
-        <v>172</v>
+        <v>0</v>
       </c>
       <c r="E73">
-        <v>72</v>
+        <v>-100</v>
       </c>
       <c r="F73" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B74">
+        <v>50</v>
+      </c>
+      <c r="C74" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D74">
+        <v>0</v>
+      </c>
+      <c r="E74">
+        <v>-50</v>
+      </c>
+      <c r="F74" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>2026-09-26</v>
+      </c>
+      <c r="B75">
+        <v>50</v>
+      </c>
+      <c r="C75" t="str">
+        <v>Vinta</v>
+      </c>
+      <c r="D75">
+        <v>242.15</v>
+      </c>
+      <c r="E75">
+        <v>192.15</v>
+      </c>
+      <c r="F75" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F75"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-27T20:34:07
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F79"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 26/09/2026</v>
+        <v>Utente: Gesss - Generato il 27/09/2026</v>
       </c>
     </row>
     <row r="3">
@@ -1899,9 +1899,89 @@
         <v/>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B76">
+        <v>50</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D76">
+        <v>0</v>
+      </c>
+      <c r="E76">
+        <v>-50</v>
+      </c>
+      <c r="F76" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B77">
+        <v>50</v>
+      </c>
+      <c r="C77" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D77">
+        <v>0</v>
+      </c>
+      <c r="E77">
+        <v>-50</v>
+      </c>
+      <c r="F77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B78">
+        <v>50</v>
+      </c>
+      <c r="C78" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D78">
+        <v>0</v>
+      </c>
+      <c r="E78">
+        <v>-50</v>
+      </c>
+      <c r="F78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>2026-09-27</v>
+      </c>
+      <c r="B79">
+        <v>63</v>
+      </c>
+      <c r="C79" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D79">
+        <v>0</v>
+      </c>
+      <c r="E79">
+        <v>-63</v>
+      </c>
+      <c r="F79" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F75"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F79"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-29T14:31:15
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F81"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 27/09/2026</v>
+        <v>Utente: Gesss - Generato il 29/09/2026</v>
       </c>
     </row>
     <row r="3">
@@ -1979,9 +1979,49 @@
         <v/>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B80">
+        <v>100</v>
+      </c>
+      <c r="C80" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D80">
+        <v>0</v>
+      </c>
+      <c r="E80">
+        <v>-100</v>
+      </c>
+      <c r="F80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="B81">
+        <v>50</v>
+      </c>
+      <c r="C81" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D81">
+        <v>0</v>
+      </c>
+      <c r="E81">
+        <v>-50</v>
+      </c>
+      <c r="F81" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F79"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F81"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-29T20:29:31
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F82"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2019,9 +2019,29 @@
         <v/>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B82">
+        <v>50</v>
+      </c>
+      <c r="C82" t="str">
+        <v>Vinta</v>
+      </c>
+      <c r="D82">
+        <v>110</v>
+      </c>
+      <c r="E82">
+        <v>60</v>
+      </c>
+      <c r="F82" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F81"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F82"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-09-29T20:43:21
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F82"/>
+  <dimension ref="A1:F83"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2039,9 +2039,29 @@
         <v/>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>2026-09-29</v>
+      </c>
+      <c r="B83">
+        <v>50</v>
+      </c>
+      <c r="C83" t="str">
+        <v>Vinta</v>
+      </c>
+      <c r="D83">
+        <v>459.99</v>
+      </c>
+      <c r="E83">
+        <v>409.99</v>
+      </c>
+      <c r="F83" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F82"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F83"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-01T20:47:51
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F83"/>
+  <dimension ref="A1:F84"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 29/09/2026</v>
+        <v>Utente: Gesss - Generato il 01/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2059,9 +2059,29 @@
         <v/>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>2026-10-01</v>
+      </c>
+      <c r="B84">
+        <v>50</v>
+      </c>
+      <c r="C84" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D84">
+        <v>0</v>
+      </c>
+      <c r="E84">
+        <v>-50</v>
+      </c>
+      <c r="F84" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F83"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F84"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-03T17:59:37
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:F87"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 01/10/2026</v>
+        <v>Utente: Gesss - Generato il 03/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2079,9 +2079,69 @@
         <v/>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>2026-10-02</v>
+      </c>
+      <c r="B85">
+        <v>50</v>
+      </c>
+      <c r="C85" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85">
+        <v>-50</v>
+      </c>
+      <c r="F85" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B86">
+        <v>50</v>
+      </c>
+      <c r="C86" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D86">
+        <v>0</v>
+      </c>
+      <c r="E86">
+        <v>-50</v>
+      </c>
+      <c r="F86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>2026-10-03</v>
+      </c>
+      <c r="B87">
+        <v>50</v>
+      </c>
+      <c r="C87" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D87">
+        <v>0</v>
+      </c>
+      <c r="E87">
+        <v>-50</v>
+      </c>
+      <c r="F87" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F84"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F87"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-05T10:06:55
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F91"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 03/10/2026</v>
+        <v>Utente: Gesss - Generato il 05/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2139,9 +2139,89 @@
         <v/>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B88">
+        <v>40</v>
+      </c>
+      <c r="C88" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D88">
+        <v>0</v>
+      </c>
+      <c r="E88">
+        <v>-40</v>
+      </c>
+      <c r="F88" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B89">
+        <v>20</v>
+      </c>
+      <c r="C89" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D89">
+        <v>0</v>
+      </c>
+      <c r="E89">
+        <v>-20</v>
+      </c>
+      <c r="F89" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B90">
+        <v>40</v>
+      </c>
+      <c r="C90" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D90">
+        <v>0</v>
+      </c>
+      <c r="E90">
+        <v>-40</v>
+      </c>
+      <c r="F90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>2026-10-04</v>
+      </c>
+      <c r="B91">
+        <v>20</v>
+      </c>
+      <c r="C91" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D91">
+        <v>0</v>
+      </c>
+      <c r="E91">
+        <v>-20</v>
+      </c>
+      <c r="F91" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F87"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F91"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-06T09:44:55
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F94"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 05/10/2026</v>
+        <v>Utente: Gesss - Generato il 06/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2219,9 +2219,69 @@
         <v/>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>2026-10-05</v>
+      </c>
+      <c r="B92">
+        <v>20</v>
+      </c>
+      <c r="C92" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D92">
+        <v>0</v>
+      </c>
+      <c r="E92">
+        <v>-20</v>
+      </c>
+      <c r="F92" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>2026-10-05</v>
+      </c>
+      <c r="B93">
+        <v>40</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93">
+        <v>-40</v>
+      </c>
+      <c r="F93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>2026-10-05</v>
+      </c>
+      <c r="B94">
+        <v>50</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94">
+        <v>-50</v>
+      </c>
+      <c r="F94" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F91"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F94"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-11T20:49:11
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F92"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 06/10/2026</v>
+        <v>Utente: Gesss - Generato il 11/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -1604,7 +1604,7 @@
         <v>2026-09-19</v>
       </c>
       <c r="B61">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C61" t="str">
         <v>Persa</v>
@@ -1613,7 +1613,7 @@
         <v>0</v>
       </c>
       <c r="E61">
-        <v>-50</v>
+        <v>-100</v>
       </c>
       <c r="F61" t="str">
         <v/>
@@ -1621,10 +1621,10 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>2026-09-19</v>
+        <v>2026-09-20</v>
       </c>
       <c r="B62">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C62" t="str">
         <v>Persa</v>
@@ -1633,7 +1633,7 @@
         <v>0</v>
       </c>
       <c r="E62">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="F62" t="str">
         <v/>
@@ -1641,10 +1641,10 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="B63">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="C63" t="str">
         <v>Persa</v>
@@ -1653,7 +1653,7 @@
         <v>0</v>
       </c>
       <c r="E63">
-        <v>-50</v>
+        <v>-66</v>
       </c>
       <c r="F63" t="str">
         <v/>
@@ -1661,19 +1661,19 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-21</v>
       </c>
       <c r="B64">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="C64" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D64">
-        <v>0</v>
+        <v>598.16</v>
       </c>
       <c r="E64">
-        <v>-50</v>
+        <v>398.15999999999997</v>
       </c>
       <c r="F64" t="str">
         <v/>
@@ -1681,7 +1681,7 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-25</v>
       </c>
       <c r="B65">
         <v>50</v>
@@ -1701,19 +1701,19 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-25</v>
       </c>
       <c r="B66">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C66" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D66">
-        <v>0</v>
+        <v>172</v>
       </c>
       <c r="E66">
-        <v>-50</v>
+        <v>72</v>
       </c>
       <c r="F66" t="str">
         <v/>
@@ -1721,10 +1721,10 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>2026-09-20</v>
+        <v>2026-09-26</v>
       </c>
       <c r="B67">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C67" t="str">
         <v>Persa</v>
@@ -1733,7 +1733,7 @@
         <v>0</v>
       </c>
       <c r="E67">
-        <v>-50</v>
+        <v>-100</v>
       </c>
       <c r="F67" t="str">
         <v/>
@@ -1741,10 +1741,10 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>2026-09-21</v>
+        <v>2026-09-26</v>
       </c>
       <c r="B68">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="C68" t="str">
         <v>Persa</v>
@@ -1753,7 +1753,7 @@
         <v>0</v>
       </c>
       <c r="E68">
-        <v>-66</v>
+        <v>-50</v>
       </c>
       <c r="F68" t="str">
         <v/>
@@ -1761,19 +1761,19 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>2026-09-21</v>
+        <v>2026-09-26</v>
       </c>
       <c r="B69">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="C69" t="str">
         <v>Vinta</v>
       </c>
       <c r="D69">
-        <v>598.16</v>
+        <v>242.15</v>
       </c>
       <c r="E69">
-        <v>398.15999999999997</v>
+        <v>192.15</v>
       </c>
       <c r="F69" t="str">
         <v/>
@@ -1781,7 +1781,7 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>2026-09-25</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B70">
         <v>50</v>
@@ -1801,10 +1801,10 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>2026-09-25</v>
+        <v>2026-09-27</v>
       </c>
       <c r="B71">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="C71" t="str">
         <v>Persa</v>
@@ -1813,7 +1813,7 @@
         <v>0</v>
       </c>
       <c r="E71">
-        <v>-50</v>
+        <v>-63</v>
       </c>
       <c r="F71" t="str">
         <v/>
@@ -1821,19 +1821,19 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>2026-09-25</v>
+        <v>2026-09-28</v>
       </c>
       <c r="B72">
         <v>100</v>
       </c>
       <c r="C72" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D72">
-        <v>172</v>
+        <v>0</v>
       </c>
       <c r="E72">
-        <v>72</v>
+        <v>-100</v>
       </c>
       <c r="F72" t="str">
         <v/>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-28</v>
       </c>
       <c r="B73">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C73" t="str">
         <v>Persa</v>
@@ -1853,7 +1853,7 @@
         <v>0</v>
       </c>
       <c r="E73">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="F73" t="str">
         <v/>
@@ -1861,19 +1861,19 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>2026-09-26</v>
+        <v>2026-09-29</v>
       </c>
       <c r="B74">
         <v>50</v>
       </c>
       <c r="C74" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D74">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E74">
-        <v>-50</v>
+        <v>60</v>
       </c>
       <c r="F74" t="str">
         <v/>
@@ -1881,19 +1881,19 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>2026-09-26</v>
+        <v>2026-10-01</v>
       </c>
       <c r="B75">
         <v>50</v>
       </c>
       <c r="C75" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D75">
-        <v>242.15</v>
+        <v>0</v>
       </c>
       <c r="E75">
-        <v>192.15</v>
+        <v>-50</v>
       </c>
       <c r="F75" t="str">
         <v/>
@@ -1901,7 +1901,7 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>2026-09-27</v>
+        <v>2026-10-02</v>
       </c>
       <c r="B76">
         <v>50</v>
@@ -1921,7 +1921,7 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>2026-09-27</v>
+        <v>2026-10-03</v>
       </c>
       <c r="B77">
         <v>50</v>
@@ -1941,10 +1941,10 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>2026-09-27</v>
+        <v>2026-10-04</v>
       </c>
       <c r="B78">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C78" t="str">
         <v>Persa</v>
@@ -1953,7 +1953,7 @@
         <v>0</v>
       </c>
       <c r="E78">
-        <v>-50</v>
+        <v>-40</v>
       </c>
       <c r="F78" t="str">
         <v/>
@@ -1961,10 +1961,10 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>2026-09-27</v>
+        <v>2026-10-04</v>
       </c>
       <c r="B79">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="C79" t="str">
         <v>Persa</v>
@@ -1973,7 +1973,7 @@
         <v>0</v>
       </c>
       <c r="E79">
-        <v>-63</v>
+        <v>-20</v>
       </c>
       <c r="F79" t="str">
         <v/>
@@ -1981,10 +1981,10 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>2026-09-28</v>
+        <v>2026-10-05</v>
       </c>
       <c r="B80">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="C80" t="str">
         <v>Persa</v>
@@ -1993,7 +1993,7 @@
         <v>0</v>
       </c>
       <c r="E80">
-        <v>-100</v>
+        <v>-20</v>
       </c>
       <c r="F80" t="str">
         <v/>
@@ -2001,10 +2001,10 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>2026-09-28</v>
+        <v>2026-10-05</v>
       </c>
       <c r="B81">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C81" t="str">
         <v>Persa</v>
@@ -2013,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="E81">
-        <v>-50</v>
+        <v>-40</v>
       </c>
       <c r="F81" t="str">
         <v/>
@@ -2021,19 +2021,19 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>2026-09-29</v>
+        <v>2026-10-05</v>
       </c>
       <c r="B82">
         <v>50</v>
       </c>
       <c r="C82" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D82">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="E82">
-        <v>60</v>
+        <v>-50</v>
       </c>
       <c r="F82" t="str">
         <v/>
@@ -2041,19 +2041,19 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>2026-09-29</v>
+        <v>2026-10-09</v>
       </c>
       <c r="B83">
         <v>50</v>
       </c>
       <c r="C83" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D83">
-        <v>459.99</v>
+        <v>0</v>
       </c>
       <c r="E83">
-        <v>409.99</v>
+        <v>-50</v>
       </c>
       <c r="F83" t="str">
         <v/>
@@ -2061,7 +2061,7 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>2026-10-01</v>
+        <v>2026-10-09</v>
       </c>
       <c r="B84">
         <v>50</v>
@@ -2081,19 +2081,19 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2026-10-02</v>
+        <v>2026-10-09</v>
       </c>
       <c r="B85">
         <v>50</v>
       </c>
       <c r="C85" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D85">
-        <v>0</v>
+        <v>144.92</v>
       </c>
       <c r="E85">
-        <v>-50</v>
+        <v>94.91999999999999</v>
       </c>
       <c r="F85" t="str">
         <v/>
@@ -2101,7 +2101,7 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-10</v>
       </c>
       <c r="B86">
         <v>50</v>
@@ -2121,19 +2121,19 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>2026-10-03</v>
+        <v>2026-10-10</v>
       </c>
       <c r="B87">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C87" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D87">
-        <v>0</v>
+        <v>159.57</v>
       </c>
       <c r="E87">
-        <v>-50</v>
+        <v>104.57</v>
       </c>
       <c r="F87" t="str">
         <v/>
@@ -2141,19 +2141,19 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>2026-10-04</v>
+        <v>2026-10-10</v>
       </c>
       <c r="B88">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C88" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D88">
-        <v>0</v>
+        <v>268.72</v>
       </c>
       <c r="E88">
-        <v>-40</v>
+        <v>218.72000000000003</v>
       </c>
       <c r="F88" t="str">
         <v/>
@@ -2161,19 +2161,19 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>2026-10-04</v>
+        <v>2026-10-10</v>
       </c>
       <c r="B89">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="C89" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D89">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="E89">
-        <v>-20</v>
+        <v>49</v>
       </c>
       <c r="F89" t="str">
         <v/>
@@ -2181,10 +2181,10 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2026-10-04</v>
+        <v>2026-10-10</v>
       </c>
       <c r="B90">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C90" t="str">
         <v>Persa</v>
@@ -2193,7 +2193,7 @@
         <v>0</v>
       </c>
       <c r="E90">
-        <v>-40</v>
+        <v>-50</v>
       </c>
       <c r="F90" t="str">
         <v/>
@@ -2201,10 +2201,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2026-10-04</v>
+        <v>2026-10-10</v>
       </c>
       <c r="B91">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C91" t="str">
         <v>Persa</v>
@@ -2213,7 +2213,7 @@
         <v>0</v>
       </c>
       <c r="E91">
-        <v>-20</v>
+        <v>-50</v>
       </c>
       <c r="F91" t="str">
         <v/>
@@ -2221,10 +2221,10 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2026-10-05</v>
+        <v>2026-10-10</v>
       </c>
       <c r="B92">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="C92" t="str">
         <v>Persa</v>
@@ -2233,55 +2233,15 @@
         <v>0</v>
       </c>
       <c r="E92">
-        <v>-20</v>
+        <v>-250</v>
       </c>
       <c r="F92" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="str">
-        <v>2026-10-05</v>
-      </c>
-      <c r="B93">
-        <v>40</v>
-      </c>
-      <c r="C93" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D93">
-        <v>0</v>
-      </c>
-      <c r="E93">
-        <v>-40</v>
-      </c>
-      <c r="F93" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="str">
-        <v>2026-10-05</v>
-      </c>
-      <c r="B94">
-        <v>50</v>
-      </c>
-      <c r="C94" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D94">
-        <v>0</v>
-      </c>
-      <c r="E94">
-        <v>-50</v>
-      </c>
-      <c r="F94" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F92"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-12T20:10:40
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F94"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 11/10/2026</v>
+        <v>Utente: Gesss - Generato il 12/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2239,9 +2239,49 @@
         <v/>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>2026-10-12</v>
+      </c>
+      <c r="B93">
+        <v>50</v>
+      </c>
+      <c r="C93" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D93">
+        <v>0</v>
+      </c>
+      <c r="E93">
+        <v>-50</v>
+      </c>
+      <c r="F93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>2026-10-12</v>
+      </c>
+      <c r="B94">
+        <v>67</v>
+      </c>
+      <c r="C94" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D94">
+        <v>0</v>
+      </c>
+      <c r="E94">
+        <v>-67</v>
+      </c>
+      <c r="F94" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F94"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-13T20:45:42
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F94"/>
+  <dimension ref="A1:F95"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 12/10/2026</v>
+        <v>Utente: Gesss - Generato il 13/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2279,9 +2279,29 @@
         <v/>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B95">
+        <v>100</v>
+      </c>
+      <c r="C95" t="str">
+        <v>Vinta</v>
+      </c>
+      <c r="D95">
+        <v>194</v>
+      </c>
+      <c r="E95">
+        <v>94</v>
+      </c>
+      <c r="F95" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F94"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F95"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-14T20:56:28
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F95"/>
+  <dimension ref="A1:F97"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 13/10/2026</v>
+        <v>Utente: Gesss - Generato il 14/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2299,9 +2299,49 @@
         <v/>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="B96">
+        <v>50</v>
+      </c>
+      <c r="C96" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96">
+        <v>-50</v>
+      </c>
+      <c r="F96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>2026-10-14</v>
+      </c>
+      <c r="B97">
+        <v>50</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Vinta</v>
+      </c>
+      <c r="D97">
+        <v>302.03</v>
+      </c>
+      <c r="E97">
+        <v>252.02999999999997</v>
+      </c>
+      <c r="F97" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F95"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F97"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-15T19:50:27
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F98"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 14/10/2026</v>
+        <v>Utente: Gesss - Generato il 15/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2339,9 +2339,29 @@
         <v/>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>2026-10-15</v>
+      </c>
+      <c r="B98">
+        <v>50</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Vinta</v>
+      </c>
+      <c r="D98">
+        <v>116.27</v>
+      </c>
+      <c r="E98">
+        <v>66.27</v>
+      </c>
+      <c r="F98" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F97"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F98"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-15T20:48:36
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F98"/>
+  <dimension ref="A1:F99"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2359,9 +2359,29 @@
         <v/>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>2026-10-15</v>
+      </c>
+      <c r="B99">
+        <v>50</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D99">
+        <v>0</v>
+      </c>
+      <c r="E99">
+        <v>-50</v>
+      </c>
+      <c r="F99" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F99"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-15T20:51:56
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -2367,13 +2367,13 @@
         <v>50</v>
       </c>
       <c r="C99" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D99">
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="E99">
-        <v>-50</v>
+        <v>80</v>
       </c>
       <c r="F99" t="str">
         <v/>

</xml_diff>

<commit_message>
Update Gesss - 2026-10-16T02:56:03
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F100"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 15/10/2026</v>
+        <v>Utente: Gesss - Generato il 16/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2379,9 +2379,29 @@
         <v/>
       </c>
     </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="B100">
+        <v>911.75</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D100">
+        <v>0</v>
+      </c>
+      <c r="E100">
+        <v>-911.75</v>
+      </c>
+      <c r="F100" t="str">
+        <v>Ritirato</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F99"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F100"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-16T03:14:34
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -2387,16 +2387,16 @@
         <v>911.75</v>
       </c>
       <c r="C100" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D100">
-        <v>0</v>
-      </c>
-      <c r="E100">
-        <v>-911.75</v>
+        <v>PRELIEVO</v>
+      </c>
+      <c r="D100" t="str">
+        <v/>
+      </c>
+      <c r="E100" t="str">
+        <v/>
       </c>
       <c r="F100" t="str">
-        <v>Ritirato</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Gesss - 2026-10-17T20:42:58
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F104"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 16/10/2026</v>
+        <v>Utente: Gesss - Generato il 17/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2381,27 +2381,107 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="B100">
+        <v>100</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D100">
+        <v>0</v>
+      </c>
+      <c r="E100">
+        <v>-100</v>
+      </c>
+      <c r="F100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="B101">
+        <v>50</v>
+      </c>
+      <c r="C101" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D101">
+        <v>0</v>
+      </c>
+      <c r="E101">
+        <v>-50</v>
+      </c>
+      <c r="F101" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="B102">
+        <v>20</v>
+      </c>
+      <c r="C102" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D102">
+        <v>0</v>
+      </c>
+      <c r="E102">
+        <v>-20</v>
+      </c>
+      <c r="F102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="B103">
+        <v>10</v>
+      </c>
+      <c r="C103" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D103">
+        <v>0</v>
+      </c>
+      <c r="E103">
+        <v>-10</v>
+      </c>
+      <c r="F103" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
         <v>2026-10-16</v>
       </c>
-      <c r="B100">
+      <c r="B104">
         <v>911.75</v>
       </c>
-      <c r="C100" t="str">
+      <c r="C104" t="str">
         <v>PRELIEVO</v>
       </c>
-      <c r="D100" t="str">
-        <v/>
-      </c>
-      <c r="E100" t="str">
-        <v/>
-      </c>
-      <c r="F100" t="str">
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v/>
+      </c>
+      <c r="F104" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F100"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F104"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-17T20:45:28
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:F105"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2479,9 +2479,29 @@
         <v/>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="B105">
+        <v>262.5</v>
+      </c>
+      <c r="C105" t="str">
+        <v>PRELIEVO</v>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105" t="str">
+        <v/>
+      </c>
+      <c r="F105" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F104"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F105"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-18T18:23:34
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F109"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 17/10/2026</v>
+        <v>Utente: Gesss - Generato il 18/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2461,19 +2461,19 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2026-10-16</v>
+        <v>2026-10-18</v>
       </c>
       <c r="B104">
-        <v>911.75</v>
+        <v>50</v>
       </c>
       <c r="C104" t="str">
-        <v>PRELIEVO</v>
-      </c>
-      <c r="D104" t="str">
-        <v/>
-      </c>
-      <c r="E104" t="str">
-        <v/>
+        <v>Persa</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104">
+        <v>-50</v>
       </c>
       <c r="F104" t="str">
         <v/>
@@ -2481,27 +2481,107 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
+        <v>2026-10-18</v>
+      </c>
+      <c r="B105">
+        <v>50</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105">
+        <v>-50</v>
+      </c>
+      <c r="F105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>2026-10-18</v>
+      </c>
+      <c r="B106">
+        <v>50</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D106">
+        <v>0</v>
+      </c>
+      <c r="E106">
+        <v>-50</v>
+      </c>
+      <c r="F106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>2026-10-18</v>
+      </c>
+      <c r="B107">
+        <v>100</v>
+      </c>
+      <c r="C107" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D107">
+        <v>0</v>
+      </c>
+      <c r="E107">
+        <v>-100</v>
+      </c>
+      <c r="F107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="B108">
+        <v>911.75</v>
+      </c>
+      <c r="C108" t="str">
+        <v>PRELIEVO</v>
+      </c>
+      <c r="D108" t="str">
+        <v/>
+      </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
+      <c r="F108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
         <v>2026-10-17</v>
       </c>
-      <c r="B105">
+      <c r="B109">
         <v>262.5</v>
       </c>
-      <c r="C105" t="str">
+      <c r="C109" t="str">
         <v>PRELIEVO</v>
       </c>
-      <c r="D105" t="str">
-        <v/>
-      </c>
-      <c r="E105" t="str">
-        <v/>
-      </c>
-      <c r="F105" t="str">
+      <c r="D109" t="str">
+        <v/>
+      </c>
+      <c r="E109" t="str">
+        <v/>
+      </c>
+      <c r="F109" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F109"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-19T21:03:30
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F105"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 18/10/2026</v>
+        <v>Utente: Gesss - Generato il 19/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2067,13 +2067,13 @@
         <v>50</v>
       </c>
       <c r="C84" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D84">
-        <v>0</v>
+        <v>144.92</v>
       </c>
       <c r="E84">
-        <v>-50</v>
+        <v>94.91999999999999</v>
       </c>
       <c r="F84" t="str">
         <v/>
@@ -2081,19 +2081,19 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>2026-10-09</v>
+        <v>2026-10-10</v>
       </c>
       <c r="B85">
         <v>50</v>
       </c>
       <c r="C85" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D85">
-        <v>144.92</v>
+        <v>0</v>
       </c>
       <c r="E85">
-        <v>94.91999999999999</v>
+        <v>-50</v>
       </c>
       <c r="F85" t="str">
         <v/>
@@ -2104,16 +2104,16 @@
         <v>2026-10-10</v>
       </c>
       <c r="B86">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C86" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D86">
-        <v>0</v>
+        <v>159.57</v>
       </c>
       <c r="E86">
-        <v>-50</v>
+        <v>104.57</v>
       </c>
       <c r="F86" t="str">
         <v/>
@@ -2124,16 +2124,16 @@
         <v>2026-10-10</v>
       </c>
       <c r="B87">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C87" t="str">
         <v>Vinta</v>
       </c>
       <c r="D87">
-        <v>159.57</v>
+        <v>268.72</v>
       </c>
       <c r="E87">
-        <v>104.57</v>
+        <v>218.72000000000003</v>
       </c>
       <c r="F87" t="str">
         <v/>
@@ -2144,16 +2144,16 @@
         <v>2026-10-10</v>
       </c>
       <c r="B88">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C88" t="str">
         <v>Vinta</v>
       </c>
       <c r="D88">
-        <v>268.72</v>
+        <v>149</v>
       </c>
       <c r="E88">
-        <v>218.72000000000003</v>
+        <v>49</v>
       </c>
       <c r="F88" t="str">
         <v/>
@@ -2164,16 +2164,16 @@
         <v>2026-10-10</v>
       </c>
       <c r="B89">
-        <v>100</v>
+        <v>250</v>
       </c>
       <c r="C89" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D89">
-        <v>149</v>
+        <v>0</v>
       </c>
       <c r="E89">
-        <v>49</v>
+        <v>-250</v>
       </c>
       <c r="F89" t="str">
         <v/>
@@ -2181,7 +2181,7 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>2026-10-10</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B90">
         <v>50</v>
@@ -2201,10 +2201,10 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>2026-10-10</v>
+        <v>2026-10-12</v>
       </c>
       <c r="B91">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="C91" t="str">
         <v>Persa</v>
@@ -2213,7 +2213,7 @@
         <v>0</v>
       </c>
       <c r="E91">
-        <v>-50</v>
+        <v>-67</v>
       </c>
       <c r="F91" t="str">
         <v/>
@@ -2221,19 +2221,19 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>2026-10-10</v>
+        <v>2026-10-13</v>
       </c>
       <c r="B92">
-        <v>250</v>
+        <v>100</v>
       </c>
       <c r="C92" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D92">
-        <v>0</v>
+        <v>194</v>
       </c>
       <c r="E92">
-        <v>-250</v>
+        <v>94</v>
       </c>
       <c r="F92" t="str">
         <v/>
@@ -2241,7 +2241,7 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-14</v>
       </c>
       <c r="B93">
         <v>50</v>
@@ -2261,19 +2261,19 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>2026-10-12</v>
+        <v>2026-10-14</v>
       </c>
       <c r="B94">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="C94" t="str">
-        <v>Persa</v>
+        <v>Vinta</v>
       </c>
       <c r="D94">
-        <v>0</v>
+        <v>302.03</v>
       </c>
       <c r="E94">
-        <v>-67</v>
+        <v>252.02999999999997</v>
       </c>
       <c r="F94" t="str">
         <v/>
@@ -2281,19 +2281,19 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>2026-10-13</v>
+        <v>2026-10-15</v>
       </c>
       <c r="B95">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C95" t="str">
         <v>Vinta</v>
       </c>
       <c r="D95">
-        <v>194</v>
+        <v>116.27</v>
       </c>
       <c r="E95">
-        <v>94</v>
+        <v>66.27</v>
       </c>
       <c r="F95" t="str">
         <v/>
@@ -2301,10 +2301,10 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>2026-10-14</v>
+        <v>2026-10-17</v>
       </c>
       <c r="B96">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C96" t="str">
         <v>Persa</v>
@@ -2313,7 +2313,7 @@
         <v>0</v>
       </c>
       <c r="E96">
-        <v>-50</v>
+        <v>-100</v>
       </c>
       <c r="F96" t="str">
         <v/>
@@ -2321,19 +2321,19 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>2026-10-14</v>
+        <v>2026-10-17</v>
       </c>
       <c r="B97">
         <v>50</v>
       </c>
       <c r="C97" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D97">
-        <v>302.03</v>
+        <v>0</v>
       </c>
       <c r="E97">
-        <v>252.02999999999997</v>
+        <v>-50</v>
       </c>
       <c r="F97" t="str">
         <v/>
@@ -2341,19 +2341,19 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-17</v>
       </c>
       <c r="B98">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="C98" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D98">
-        <v>116.27</v>
+        <v>0</v>
       </c>
       <c r="E98">
-        <v>66.27</v>
+        <v>-20</v>
       </c>
       <c r="F98" t="str">
         <v/>
@@ -2361,19 +2361,19 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>2026-10-15</v>
+        <v>2026-10-17</v>
       </c>
       <c r="B99">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="C99" t="str">
-        <v>Vinta</v>
+        <v>Persa</v>
       </c>
       <c r="D99">
-        <v>130</v>
+        <v>0</v>
       </c>
       <c r="E99">
-        <v>80</v>
+        <v>-10</v>
       </c>
       <c r="F99" t="str">
         <v/>
@@ -2381,10 +2381,10 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>2026-10-17</v>
+        <v>2026-10-18</v>
       </c>
       <c r="B100">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="C100" t="str">
         <v>Persa</v>
@@ -2393,7 +2393,7 @@
         <v>0</v>
       </c>
       <c r="E100">
-        <v>-100</v>
+        <v>-50</v>
       </c>
       <c r="F100" t="str">
         <v/>
@@ -2401,10 +2401,10 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>2026-10-17</v>
+        <v>2026-10-18</v>
       </c>
       <c r="B101">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="C101" t="str">
         <v>Persa</v>
@@ -2413,7 +2413,7 @@
         <v>0</v>
       </c>
       <c r="E101">
-        <v>-50</v>
+        <v>-100</v>
       </c>
       <c r="F101" t="str">
         <v/>
@@ -2421,10 +2421,10 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>2026-10-17</v>
+        <v>2026-10-19</v>
       </c>
       <c r="B102">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="C102" t="str">
         <v>Persa</v>
@@ -2433,7 +2433,7 @@
         <v>0</v>
       </c>
       <c r="E102">
-        <v>-20</v>
+        <v>-50</v>
       </c>
       <c r="F102" t="str">
         <v/>
@@ -2441,10 +2441,10 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>2026-10-17</v>
+        <v>2026-10-19</v>
       </c>
       <c r="B103">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="C103" t="str">
         <v>Persa</v>
@@ -2453,7 +2453,7 @@
         <v>0</v>
       </c>
       <c r="E103">
-        <v>-10</v>
+        <v>-100</v>
       </c>
       <c r="F103" t="str">
         <v/>
@@ -2461,19 +2461,19 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2026-10-18</v>
+        <v>2026-10-16</v>
       </c>
       <c r="B104">
-        <v>50</v>
+        <v>911.75</v>
       </c>
       <c r="C104" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D104">
-        <v>0</v>
-      </c>
-      <c r="E104">
-        <v>-50</v>
+        <v>PRELIEVO</v>
+      </c>
+      <c r="D104" t="str">
+        <v/>
+      </c>
+      <c r="E104" t="str">
+        <v/>
       </c>
       <c r="F104" t="str">
         <v/>
@@ -2481,107 +2481,27 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>2026-10-18</v>
+        <v>2026-10-17</v>
       </c>
       <c r="B105">
-        <v>50</v>
+        <v>262.5</v>
       </c>
       <c r="C105" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D105">
-        <v>0</v>
-      </c>
-      <c r="E105">
-        <v>-50</v>
+        <v>PRELIEVO</v>
+      </c>
+      <c r="D105" t="str">
+        <v/>
+      </c>
+      <c r="E105" t="str">
+        <v/>
       </c>
       <c r="F105" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="str">
-        <v>2026-10-18</v>
-      </c>
-      <c r="B106">
-        <v>50</v>
-      </c>
-      <c r="C106" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D106">
-        <v>0</v>
-      </c>
-      <c r="E106">
-        <v>-50</v>
-      </c>
-      <c r="F106" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="str">
-        <v>2026-10-18</v>
-      </c>
-      <c r="B107">
-        <v>100</v>
-      </c>
-      <c r="C107" t="str">
-        <v>Persa</v>
-      </c>
-      <c r="D107">
-        <v>0</v>
-      </c>
-      <c r="E107">
-        <v>-100</v>
-      </c>
-      <c r="F107" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="str">
-        <v>2026-10-16</v>
-      </c>
-      <c r="B108">
-        <v>911.75</v>
-      </c>
-      <c r="C108" t="str">
-        <v>PRELIEVO</v>
-      </c>
-      <c r="D108" t="str">
-        <v/>
-      </c>
-      <c r="E108" t="str">
-        <v/>
-      </c>
-      <c r="F108" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="str">
-        <v>2026-10-17</v>
-      </c>
-      <c r="B109">
-        <v>262.5</v>
-      </c>
-      <c r="C109" t="str">
-        <v>PRELIEVO</v>
-      </c>
-      <c r="D109" t="str">
-        <v/>
-      </c>
-      <c r="E109" t="str">
-        <v/>
-      </c>
-      <c r="F109" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F109"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F105"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-23T02:01:23
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F109"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 19/10/2026</v>
+        <v>Utente: Gesss - Generato il 23/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2461,19 +2461,19 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>2026-10-16</v>
+        <v>2026-10-22</v>
       </c>
       <c r="B104">
-        <v>911.75</v>
+        <v>50</v>
       </c>
       <c r="C104" t="str">
-        <v>PRELIEVO</v>
-      </c>
-      <c r="D104" t="str">
-        <v/>
-      </c>
-      <c r="E104" t="str">
-        <v/>
+        <v>Persa</v>
+      </c>
+      <c r="D104">
+        <v>0</v>
+      </c>
+      <c r="E104">
+        <v>-50</v>
       </c>
       <c r="F104" t="str">
         <v/>
@@ -2481,27 +2481,107 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="B105">
+        <v>50</v>
+      </c>
+      <c r="C105" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D105">
+        <v>0</v>
+      </c>
+      <c r="E105">
+        <v>-50</v>
+      </c>
+      <c r="F105" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="B106">
+        <v>70</v>
+      </c>
+      <c r="C106" t="str">
+        <v>Persa</v>
+      </c>
+      <c r="D106">
+        <v>0</v>
+      </c>
+      <c r="E106">
+        <v>-70</v>
+      </c>
+      <c r="F106" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>2026-10-16</v>
+      </c>
+      <c r="B107">
+        <v>911.75</v>
+      </c>
+      <c r="C107" t="str">
+        <v>PRELIEVO</v>
+      </c>
+      <c r="D107" t="str">
+        <v/>
+      </c>
+      <c r="E107" t="str">
+        <v/>
+      </c>
+      <c r="F107" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
         <v>2026-10-17</v>
       </c>
-      <c r="B105">
+      <c r="B108">
         <v>262.5</v>
       </c>
-      <c r="C105" t="str">
+      <c r="C108" t="str">
         <v>PRELIEVO</v>
       </c>
-      <c r="D105" t="str">
-        <v/>
-      </c>
-      <c r="E105" t="str">
-        <v/>
-      </c>
-      <c r="F105" t="str">
+      <c r="D108" t="str">
+        <v/>
+      </c>
+      <c r="E108" t="str">
+        <v/>
+      </c>
+      <c r="F108" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="B109" t="str">
+        <v/>
+      </c>
+      <c r="C109" t="str">
+        <v>DEPOSITO</v>
+      </c>
+      <c r="D109">
+        <v>150</v>
+      </c>
+      <c r="E109" t="str">
+        <v/>
+      </c>
+      <c r="F109" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F105"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F109"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-23T20:20:22
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F110"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2521,19 +2521,19 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>2026-10-16</v>
+        <v>2026-10-23</v>
       </c>
       <c r="B107">
-        <v>911.75</v>
+        <v>100</v>
       </c>
       <c r="C107" t="str">
-        <v>PRELIEVO</v>
-      </c>
-      <c r="D107" t="str">
-        <v/>
-      </c>
-      <c r="E107" t="str">
-        <v/>
+        <v>Vinta</v>
+      </c>
+      <c r="D107">
+        <v>247.07</v>
+      </c>
+      <c r="E107">
+        <v>147.07</v>
       </c>
       <c r="F107" t="str">
         <v/>
@@ -2541,10 +2541,10 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>2026-10-17</v>
+        <v>2026-10-16</v>
       </c>
       <c r="B108">
-        <v>262.5</v>
+        <v>911.75</v>
       </c>
       <c r="C108" t="str">
         <v>PRELIEVO</v>
@@ -2561,27 +2561,47 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="B109">
+        <v>262.5</v>
+      </c>
+      <c r="C109" t="str">
+        <v>PRELIEVO</v>
+      </c>
+      <c r="D109" t="str">
+        <v/>
+      </c>
+      <c r="E109" t="str">
+        <v/>
+      </c>
+      <c r="F109" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
         <v>2026-10-22</v>
       </c>
-      <c r="B109" t="str">
-        <v/>
-      </c>
-      <c r="C109" t="str">
+      <c r="B110" t="str">
+        <v/>
+      </c>
+      <c r="C110" t="str">
         <v>DEPOSITO</v>
       </c>
-      <c r="D109">
+      <c r="D110">
         <v>150</v>
       </c>
-      <c r="E109" t="str">
-        <v/>
-      </c>
-      <c r="F109" t="str">
+      <c r="E110" t="str">
+        <v/>
+      </c>
+      <c r="F110" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F109"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F110"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Gesss - 2026-10-26T06:45:54
</commit_message>
<xml_diff>
--- a/excel/gestione_Gesss.xlsx
+++ b/excel/gestione_Gesss.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F110"/>
+  <dimension ref="A1:F111"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -436,7 +436,7 @@
         <v/>
       </c>
       <c r="F2" t="str">
-        <v>Utente: Gesss - Generato il 23/10/2026</v>
+        <v>Utente: Gesss - Generato il 26/10/2026</v>
       </c>
     </row>
     <row r="3">
@@ -2541,19 +2541,19 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>2026-10-16</v>
+        <v>2026-10-26</v>
       </c>
       <c r="B108">
-        <v>911.75</v>
+        <v>11.38</v>
       </c>
       <c r="C108" t="str">
-        <v>PRELIEVO</v>
-      </c>
-      <c r="D108" t="str">
-        <v/>
-      </c>
-      <c r="E108" t="str">
-        <v/>
+        <v>Persa</v>
+      </c>
+      <c r="D108">
+        <v>0</v>
+      </c>
+      <c r="E108">
+        <v>-11.38</v>
       </c>
       <c r="F108" t="str">
         <v/>
@@ -2561,10 +2561,10 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>2026-10-17</v>
+        <v>2026-10-16</v>
       </c>
       <c r="B109">
-        <v>262.5</v>
+        <v>911.75</v>
       </c>
       <c r="C109" t="str">
         <v>PRELIEVO</v>
@@ -2581,27 +2581,47 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
+        <v>2026-10-17</v>
+      </c>
+      <c r="B110">
+        <v>262.5</v>
+      </c>
+      <c r="C110" t="str">
+        <v>PRELIEVO</v>
+      </c>
+      <c r="D110" t="str">
+        <v/>
+      </c>
+      <c r="E110" t="str">
+        <v/>
+      </c>
+      <c r="F110" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
         <v>2026-10-22</v>
       </c>
-      <c r="B110" t="str">
-        <v/>
-      </c>
-      <c r="C110" t="str">
+      <c r="B111" t="str">
+        <v/>
+      </c>
+      <c r="C111" t="str">
         <v>DEPOSITO</v>
       </c>
-      <c r="D110">
+      <c r="D111">
         <v>150</v>
       </c>
-      <c r="E110" t="str">
-        <v/>
-      </c>
-      <c r="F110" t="str">
+      <c r="E111" t="str">
+        <v/>
+      </c>
+      <c r="F111" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F110"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F111"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>